<commit_message>
docs: module tracker after the control and governance module (overall 36%)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ZOAURO_Module_Build-members.xlsx
+++ b/ZOAURO_Module_Build-members.xlsx
@@ -674,7 +674,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Progress updated 2026-10-15 from the code on main (local and GitHub). Progress % = share of the Phase 1 scope built and tested (API + screens + tests). Rows from 17 on were added from the roadmap v2 and the owner decisions of 2026-10-14.</t>
+          <t xml:space="preserve">Progress updated 2026-10-16 from the code on main (local and GitHub). Progress % = share of the Phase 1 scope built and tested (API + screens + tests). Rows from 17 on were added from the roadmap v2 and the owner decisions of 2026-10-14.</t>
         </is>
       </c>
     </row>
@@ -978,20 +978,20 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not started</t>
+          <t xml:space="preserve">In review</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">A read-only "my zones" chip exists in the top bar. Switcher designed in doc 59 (Phase 4 of the Control &amp; Governance spec).</t>
+          <t xml:space="preserve">Top-bar switcher live (f88ff40): ?zone=&lt;CODE&gt; in the URL, remembered per member, a code the member may not use falls back to all; Zonal dashboard, access requests, Platform Settings and Settings History follow it; e2e green. Left: Zone Teams, Access History and Audit Logs still filter by their own zone picker.</t>
         </is>
       </c>
       <c r="H10" s="10">
-        <v>0.1</v>
+        <v>0.85</v>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Follow-up screens</t>
         </is>
       </c>
     </row>
@@ -1388,11 +1388,11 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Super Admin and Zonal dashboards live with real data (zones, security, recent activity, my zones and limits). Order and money tiles come with those modules.</t>
+          <t xml:space="preserve">Super Admin and Zonal dashboards live with real data (zones, security, recent activity, my zones and limits; Zonal Admin counts and recent access changes added 2026-10-15). Pending access requests badge comes with R13. Order and money tiles come with those modules.</t>
         </is>
       </c>
       <c r="H19" s="10">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
@@ -1613,15 +1613,15 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner spec "Control &amp; Governance" (2026-10-15). Phase 0 plan in doc 59: default applies until the Super Admin saves a value; zone overrides; settings history. Waiting for the owner to approve the plan and decisions Q1-Q8.</t>
+          <t xml:space="preserve">Plan approved (doc 59, D109-D116). Settings API (8feb77e) and screens (8b9f507): Platform Settings with source and effect badges, edit &gt; preview &gt; reason &gt; re-auth &gt; save, reset, per-zone values; Settings History. Refund caps enforced in the access editor (D110). Migration applied to zoauro 2026-10-16; e2e change, history and reset green. Left: each remaining setting connects to its module when that module is built (Refunds, Support, Notifications, Orders, Onboarding).</t>
         </is>
       </c>
       <c r="H24" s="10">
-        <v>0.15</v>
+        <v>0.75</v>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phase 0 plan (approval)</t>
+          <t xml:space="preserve">Connect with modules</t>
         </is>
       </c>
     </row>
@@ -1788,16 +1788,16 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not started</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plan page in the menu. Builds on M03. Designed in doc 59 (Phase 4 of the Control &amp; Governance spec).</t>
+          <t xml:space="preserve">API (faff626) and screens (02d44cd): Zonal Admins ask for a zone or a permission with a reason and follow the status; the Super Admin approves (profile for a zone, reason, password) or rejects (reason); dashboard banner; no self-approval; e2e request-to-approval green.</t>
         </is>
       </c>
       <c r="H28" s="10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
@@ -2025,7 +2025,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Control &amp; Governance module: Phase 0 plan (doc 59) waits for the owner approval; then settings, access requests (R13) and the zone switcher (M05). Admin email update waits for the owner "approved". After that: Delivery Partners. Restaurants/Homemakers and Orders with the colleagues.</t>
+          <t xml:space="preserve">Control &amp; Governance module (doc 59) built: settings, settings history, access requests, zone switcher; migration applied; e2e green. Next: port the colleagues' Restaurants/Homemakers and Orders work (owner sends it EOD), then Delivery Partners.</t>
         </is>
       </c>
     </row>

</xml_diff>